<commit_message>
Add historical backfill, multi-year holiday fix, and MA breakout charts
- Fix HolidayCalendar to support multiple years (2025+2026); was silently
  producing wrong business day dates for all 2025 trade dates
- Add build_historical_dataset.py: combines Barchart Term SOFR CSVs,
  FWD_Points_Actual_Historical.xlsx, and yfinance USDSGD spot to produce
  output_historical_1m/3m/6m.xlsx (Jan 2025 – Feb 2026, ~268 rows each)
- Add plot_ma_analysis.py: merges historical + master files into
  output_combined_*.xlsx, computes 60-day MA, and produces 8 PNG charts
  (recent Oct 2025–present and full-history views, individual + 3-panel)
- Add source data files: Barchart SOFR CSVs and FWD_Points_Actual_Historical.xlsx
- Update CLAUDE.md with new scripts, data sources, and file inventory
- Add SESSION_2026-03-24.md documenting today's work and findings

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output_master_1m.xlsx
+++ b/output_master_1m.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Methodology" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1300,6 +1300,142 @@
       </c>
       <c r="J25" t="n">
         <v>-255.095859605768</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>46104</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>46135</v>
+      </c>
+      <c r="D26" t="n">
+        <v>31</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3.67672</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.2814</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-27.43</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1.278657</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1.199389577639535</v>
+      </c>
+      <c r="J26" t="n">
+        <v>-247.7330422360465</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>46136</v>
+      </c>
+      <c r="D27" t="n">
+        <v>31</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3.67504</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1.2796</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-27.5</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1.27685</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1.187671819035491</v>
+      </c>
+      <c r="J27" t="n">
+        <v>-248.7368180964509</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>46106</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>46139</v>
+      </c>
+      <c r="D28" t="n">
+        <v>33</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3.67495</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1.2816</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-29.65</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.278635</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.158483746720895</v>
+      </c>
+      <c r="J28" t="n">
+        <v>-251.6466253279105</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>46139</v>
+      </c>
+      <c r="D29" t="n">
+        <v>32</v>
+      </c>
+      <c r="E29" t="n">
+        <v>3.67786</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.2751</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-28.25</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1.272275</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1.193610917220891</v>
+      </c>
+      <c r="J29" t="n">
+        <v>-248.4249082779109</v>
       </c>
     </row>
   </sheetData>
@@ -1347,7 +1483,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -1357,7 +1493,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.130557074669068</v>
+        <v>1.138304494738372</v>
       </c>
     </row>
     <row r="5">
@@ -1367,7 +1503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.669287500000001</v>
+        <v>3.670266785714286</v>
       </c>
     </row>
     <row r="6">
@@ -1377,7 +1513,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-253.8730425330932</v>
+        <v>-253.1962290975913</v>
       </c>
     </row>
     <row r="7">
@@ -1427,7 +1563,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>29.41666666666667</v>
+        <v>29.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Hedging_Cost_bps column to pipeline and Roam output
- calculate_swap_implied_rates.py: compute Hedging_Cost_bps = (Implied_SGD_Rate - SOFR×365/360)×100 alongside existing Rate_Diff_bps
- post_to_roam.py: extend Roam block with SOFR and Hedging Cost lines (prospective)
- add_hedging_cost.py: one-time retrofit script for existing output_master_*m.xlsx files
- output_master_{1m,3m,6m}.xlsx: retrofitted with Hedging_Cost_bps column
- CLAUDE.md: documented new column, script, and Roam block format
- rollback_2026-03-28.md: rollback instructions if pipeline breaks

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output_master_1m.xlsx
+++ b/output_master_1m.xlsx
@@ -1,15 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Methodology" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,6 +483,11 @@
           <t>Rate_Diff_bps</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Hedging_Cost_bps</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -519,6 +522,9 @@
       <c r="J2" t="n">
         <v>-249.5729340830794</v>
       </c>
+      <c r="K2" t="n">
+        <v>-254.6684479719682</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -553,6 +559,9 @@
       <c r="J3" t="n">
         <v>-246.9330653696609</v>
       </c>
+      <c r="K3" t="n">
+        <v>-252.0321487029942</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -587,6 +596,9 @@
       <c r="J4" t="n">
         <v>-247.5958142800976</v>
       </c>
+      <c r="K4" t="n">
+        <v>-252.6972865023198</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -621,6 +633,9 @@
       <c r="J5" t="n">
         <v>-253.3423714180751</v>
       </c>
+      <c r="K5" t="n">
+        <v>-258.437010306964</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -655,6 +670,9 @@
       <c r="J6" t="n">
         <v>-254.4662691902107</v>
       </c>
+      <c r="K6" t="n">
+        <v>-259.5569497457663</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -689,6 +707,9 @@
       <c r="J7" t="n">
         <v>-255.4793584464259</v>
       </c>
+      <c r="K7" t="n">
+        <v>-260.5700390019815</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -723,6 +744,9 @@
       <c r="J8" t="n">
         <v>-252.0745324977909</v>
       </c>
+      <c r="K8" t="n">
+        <v>-257.1585186089019</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -757,6 +781,9 @@
       <c r="J9" t="n">
         <v>-255.4206109829415</v>
       </c>
+      <c r="K9" t="n">
+        <v>-260.5034443162748</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -791,6 +818,9 @@
       <c r="J10" t="n">
         <v>-256.5081999154748</v>
       </c>
+      <c r="K10" t="n">
+        <v>-261.5910332488081</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -825,6 +855,9 @@
       <c r="J11" t="n">
         <v>-254.2812202239006</v>
       </c>
+      <c r="K11" t="n">
+        <v>-259.3640674461228</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -859,6 +892,9 @@
       <c r="J12" t="n">
         <v>-252.4920558401689</v>
       </c>
+      <c r="K12" t="n">
+        <v>-257.5749030623911</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -893,6 +929,9 @@
       <c r="J13" t="n">
         <v>-246.1416508256062</v>
       </c>
+      <c r="K13" t="n">
+        <v>-251.2350397144951</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -927,6 +966,9 @@
       <c r="J14" t="n">
         <v>-245.7813184411759</v>
       </c>
+      <c r="K14" t="n">
+        <v>-250.8747073300648</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -961,6 +1003,9 @@
       <c r="J15" t="n">
         <v>-251.0820770370311</v>
       </c>
+      <c r="K15" t="n">
+        <v>-256.1836881481423</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -995,6 +1040,9 @@
       <c r="J16" t="n">
         <v>-281.5844514725661</v>
       </c>
+      <c r="K16" t="n">
+        <v>-286.6868542503439</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1029,6 +1077,9 @@
       <c r="J17" t="n">
         <v>-247.2692513715374</v>
       </c>
+      <c r="K17" t="n">
+        <v>-252.375418038204</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1063,6 +1114,9 @@
       <c r="J18" t="n">
         <v>-228.4541093142201</v>
       </c>
+      <c r="K18" t="n">
+        <v>-233.555498203109</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1097,6 +1151,9 @@
       <c r="J19" t="n">
         <v>-259.7031984433297</v>
       </c>
+      <c r="K19" t="n">
+        <v>-264.7967539988852</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1131,6 +1188,9 @@
       <c r="J20" t="n">
         <v>-260.2650658082209</v>
       </c>
+      <c r="K20" t="n">
+        <v>-265.3622324748874</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1165,6 +1225,9 @@
       <c r="J21" t="n">
         <v>-259.8863805824694</v>
       </c>
+      <c r="K21" t="n">
+        <v>-264.9925750269138</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1199,6 +1262,9 @@
       <c r="J22" t="n">
         <v>-262.703146576207</v>
       </c>
+      <c r="K22" t="n">
+        <v>-267.8025493539848</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1233,6 +1299,9 @@
       <c r="J23" t="n">
         <v>-255.6648561027384</v>
       </c>
+      <c r="K23" t="n">
+        <v>-260.7733561027383</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1267,6 +1336,9 @@
       <c r="J24" t="n">
         <v>-261.1552229655416</v>
       </c>
+      <c r="K24" t="n">
+        <v>-266.2637229655415</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1301,6 +1373,9 @@
       <c r="J25" t="n">
         <v>-255.095859605768</v>
       </c>
+      <c r="K25" t="n">
+        <v>-260.206359605768</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1335,6 +1410,9 @@
       <c r="J26" t="n">
         <v>-247.7330422360465</v>
       </c>
+      <c r="K26" t="n">
+        <v>-252.839597791602</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1369,6 +1447,9 @@
       <c r="J27" t="n">
         <v>-248.7368180964509</v>
       </c>
+      <c r="K27" t="n">
+        <v>-253.8410403186732</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1403,6 +1484,9 @@
       <c r="J28" t="n">
         <v>-251.6466253279105</v>
       </c>
+      <c r="K28" t="n">
+        <v>-256.7507225501327</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1437,210 +1521,156 @@
       <c r="J29" t="n">
         <v>-248.4249082779109</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1M</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Number of Trades</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Average Implied SGD Rate 1M (%)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1.138304494738372</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Average USD SOFR 1M (%)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3.670266785714286</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Average Rate Differential (bps)</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>-253.1962290975913</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Min Implied SGD Rate 1M (%)</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.8578854852743394</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Max Implied SGD Rate 1M (%)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1.388458906857799</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Min Days</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Max Days</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Average Days</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>29.75</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Methodology</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
-USD/SGD FX SWAP IMPLIED RATE CALCULATION METHODOLOGY
-TENOR: 1M (1 months)
-1. BUSINESS DAY CALCULATION (T+2)
-   - Both US and Singapore markets must be open
-   - US holidays: NY SIFMA banking calendar
-   - Singapore holidays: MOM official public holidays
-   - Spot Date = Trade Date + 2 business days
-2. FORWARD DATE CALCULATION (1M)
-   - Convention: Same day 1 month(s) later, adjusted to business day
-   - Following business day convention if falls on holiday/weekend
-   - Handles month-end adjustments (e.g., Jan 31 → Feb 28)
-3. DAY COUNT CONVENTIONS
-   - USD (SOFR): ACT/360 (Actual days / 360)
-   - SGD: ACT/365 (Actual days / 365)
-4. COVERED INTEREST PARITY (CIP) FORMULA
-   F = S × (1 + r_SGD × days/365) / (1 + r_USD × days/360)
-   Solving for implied SGD rate:
-   r_SGD = [(F/S) × (1 + r_USD × days/360) - 1] × (365/days)
-   Where:
-   - F = Forward FX rate (SGD per USD)
-   - S = Spot FX rate (SGD per USD)
-   - r_SGD = Singapore Dollar interest rate (solving for)
-   - r_USD = US Dollar interest rate (1M Term SOFR)
-   - days = Actual calendar days between spot and forward
-5. FORWARD RATE CALCULATION
-   Forward Rate = Spot Rate + (Forward Points / 10,000)
-   Note: 1 pip = 0.0001
-6. TENOR-SPECIFIC PARAMETERS
-   - 1M: ~28-31 days (spot + 1 month)
-   - 3M: ~89-92 days (spot + 3 months)
-   - 6M: ~181-184 days (spot + 6 months)
-   Actual days vary based on:
-   - Calendar month lengths
-   - Business day adjustments
-   - Holiday patterns
-7. DATA SOURCES
-   - US Holidays: NY SIFMA
-   - Singapore Holidays: Ministry of Manpower (MOM)
-   - URL: https://www.mom.gov.sg/employment-practices/public-holidays
-   - Term SOFR: CME Group
-8. RATE DIFFERENTIAL
-   Differential (bps) = (Implied SGD Rate - USD SOFR Rate) × 100
-   Negative differential indicates SGD rates are lower than USD rates
-9. ECONOMIC INTERPRETATION
-   - Negative forward points → SGD appreciation expected
-   - Lower SGD rates → Reflects MAS exchange rate policy
-   - Rate differential → Carry trade opportunity
-   - Longer tenors → Larger accumulated differential
-        </t>
-        </is>
+      <c r="K29" t="n">
+        <v>-253.5330471667997</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>46139</v>
+      </c>
+      <c r="D30" t="n">
+        <v>31</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3.67855</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.2786</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-27.5</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1.27585</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1.189237610357607</v>
+      </c>
+      <c r="J30" t="n">
+        <v>-248.9312389642392</v>
+      </c>
+      <c r="K30" t="n">
+        <v>-254.0403361864615</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>46111</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="D31" t="n">
+        <v>31</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3.68065</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.2806</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-27.36</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1.277864</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1.208242512823935</v>
+      </c>
+      <c r="J31" t="n">
+        <v>-247.2407487176065</v>
+      </c>
+      <c r="K31" t="n">
+        <v>-252.3527626064954</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>46112</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="D32" t="n">
+        <v>30</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3.67636</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.2846</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-26.5</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1.28195</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1.209870866050074</v>
+      </c>
+      <c r="J32" t="n">
+        <v>-246.6489133949926</v>
+      </c>
+      <c r="K32" t="n">
+        <v>-251.7549689505481</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>46112</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="D33" t="n">
+        <v>30</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3.67306</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.2876</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-26.815</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1.2849185</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1.18254181368365</v>
+      </c>
+      <c r="J33" t="n">
+        <v>-249.051818631635</v>
+      </c>
+      <c r="K33" t="n">
+        <v>-254.1532908538572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>